<commit_message>
Māori Maps waka citations: Araiteuru, Uruao, Nukutaimemeha, Tereānini, Matawhaorua, Tauira, Tauira-mai-tawhiti, Nukutere, Te Awatea
</commit_message>
<xml_diff>
--- a/TKM_Iwi_Hapu_Marae_Database.xlsx
+++ b/TKM_Iwi_Hapu_Marae_Database.xlsx
@@ -377,7 +377,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13823" uniqueCount="3412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14267" uniqueCount="3492">
   <si>
     <t xml:space="preserve">TKM Iwi / Hapū / Marae Database</t>
   </si>
@@ -10484,6 +10484,246 @@
   </si>
   <si>
     <t xml:space="preserve">Ngāti Te Maunga</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1283</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Araiteuru</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://maorimaps.com/en/waka/araiteuru</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1340</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1341</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moeraki</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1342</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1343</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1344</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1345</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arahura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uruao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://maorimaps.com/en/waka/uruao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1346</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1347</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1348</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1349</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1350</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ōtākou</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1351</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Te Ruahikihiki</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1352</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1353</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1354</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Te Tauraka Waka a Māui</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1355</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kāti Māhaki ki Makaawhio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1356</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1357</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wairewa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1358</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ngāti Irakēhu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waitaha, Ngati Mamoe, Ngāi Tahu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Māori Maps writes 'Ngāti Irakēhu (Waitaha, Ngati Mamoe, Ngāi Tahu)'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1359</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nukutaimemeha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://maorimaps.com/en/waka/nukutaimemeha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1360</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1361</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1362</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uepōhatu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1363</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1364</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1365</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tereānini</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://maorimaps.com/en/waka/tereānini</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1366</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1367</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1368</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1369</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matawhaorua</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://maorimaps.com/en/waka/matawhaorua</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1370</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tauira</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://maorimaps.com/en/waka/tauira</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1371</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tauira-mai-tawhiti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://maorimaps.com/en/waka/tauira-mai-tawhiti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1372</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1373</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1374</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1375</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1376</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1377</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1378</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1379</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1380</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nukutere</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://maorimaps.com/en/waka/nukutere</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1381</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1382</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1383</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1384</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1385</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1386</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://maorimaps.com/en/waka/tauria-mai-tawhiti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Māori Maps variant page "Tauria-mai-tawhiti" (typo for Tauira-mai-tawhiti)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1387</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Te Awatea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://maorimaps.com/en/waka/te-awatea</t>
   </si>
   <si>
     <t xml:space="preserve">alias_id</t>
@@ -10887,8 +11127,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Claim" displayName="Claim" ref="A1:L1339" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:L1339"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Claim" displayName="Claim" ref="A1:L1388" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:L1388"/>
   <tableColumns count="12">
     <tableColumn id="1" name="claim_id"/>
     <tableColumn id="2" name="source_id"/>
@@ -13130,7 +13370,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L1339"/>
+  <dimension ref="A1:L1388"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="9"/>
@@ -56876,6 +57116,1580 @@
         <v>703</v>
       </c>
       <c r="L1339" s="4"/>
+    </row>
+    <row r="1340" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1340" s="4" t="s">
+        <v>3369</v>
+      </c>
+      <c r="B1340" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1340" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1340" s="4" t="s">
+        <v>2119</v>
+      </c>
+      <c r="E1340" s="4"/>
+      <c r="F1340" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1340" s="4" t="s">
+        <v>3370</v>
+      </c>
+      <c r="H1340" s="4"/>
+      <c r="I1340" s="4" t="s">
+        <v>3371</v>
+      </c>
+      <c r="J1340" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1340" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1340" s="4"/>
+    </row>
+    <row r="1341" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1341" s="4" t="s">
+        <v>3372</v>
+      </c>
+      <c r="B1341" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1341" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1341" s="4" t="s">
+        <v>2187</v>
+      </c>
+      <c r="E1341" s="4"/>
+      <c r="F1341" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1341" s="4" t="s">
+        <v>3370</v>
+      </c>
+      <c r="H1341" s="4"/>
+      <c r="I1341" s="4" t="s">
+        <v>3371</v>
+      </c>
+      <c r="J1341" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1341" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1341" s="4"/>
+    </row>
+    <row r="1342" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1342" s="4" t="s">
+        <v>3373</v>
+      </c>
+      <c r="B1342" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1342" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1342" s="4" t="s">
+        <v>3374</v>
+      </c>
+      <c r="E1342" s="4"/>
+      <c r="F1342" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1342" s="4" t="s">
+        <v>3370</v>
+      </c>
+      <c r="H1342" s="4"/>
+      <c r="I1342" s="4" t="s">
+        <v>3371</v>
+      </c>
+      <c r="J1342" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1342" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1342" s="4"/>
+    </row>
+    <row r="1343" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1343" s="4" t="s">
+        <v>3375</v>
+      </c>
+      <c r="B1343" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1343" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1343" s="4" t="s">
+        <v>2274</v>
+      </c>
+      <c r="E1343" s="4"/>
+      <c r="F1343" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1343" s="4" t="s">
+        <v>3370</v>
+      </c>
+      <c r="H1343" s="4"/>
+      <c r="I1343" s="4" t="s">
+        <v>3371</v>
+      </c>
+      <c r="J1343" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1343" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1343" s="4"/>
+    </row>
+    <row r="1344" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1344" s="4" t="s">
+        <v>3376</v>
+      </c>
+      <c r="B1344" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1344" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1344" s="4" t="s">
+        <v>2324</v>
+      </c>
+      <c r="E1344" s="4"/>
+      <c r="F1344" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1344" s="4" t="s">
+        <v>3370</v>
+      </c>
+      <c r="H1344" s="4"/>
+      <c r="I1344" s="4" t="s">
+        <v>3371</v>
+      </c>
+      <c r="J1344" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1344" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1344" s="4"/>
+    </row>
+    <row r="1345" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1345" s="4" t="s">
+        <v>3377</v>
+      </c>
+      <c r="B1345" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1345" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1345" s="4" t="s">
+        <v>2425</v>
+      </c>
+      <c r="E1345" s="4"/>
+      <c r="F1345" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1345" s="4" t="s">
+        <v>3370</v>
+      </c>
+      <c r="H1345" s="4"/>
+      <c r="I1345" s="4" t="s">
+        <v>3371</v>
+      </c>
+      <c r="J1345" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1345" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1345" s="4"/>
+    </row>
+    <row r="1346" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1346" s="4" t="s">
+        <v>3378</v>
+      </c>
+      <c r="B1346" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1346" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1346" s="4" t="s">
+        <v>3379</v>
+      </c>
+      <c r="E1346" s="4"/>
+      <c r="F1346" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1346" s="4" t="s">
+        <v>3380</v>
+      </c>
+      <c r="H1346" s="4"/>
+      <c r="I1346" s="4" t="s">
+        <v>3381</v>
+      </c>
+      <c r="J1346" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1346" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1346" s="4"/>
+    </row>
+    <row r="1347" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1347" s="4" t="s">
+        <v>3382</v>
+      </c>
+      <c r="B1347" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1347" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1347" s="4" t="s">
+        <v>3379</v>
+      </c>
+      <c r="E1347" s="4"/>
+      <c r="F1347" s="4" t="s">
+        <v>700</v>
+      </c>
+      <c r="G1347" s="4" t="s">
+        <v>3286</v>
+      </c>
+      <c r="H1347" s="4"/>
+      <c r="I1347" s="4" t="s">
+        <v>3381</v>
+      </c>
+      <c r="J1347" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1347" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1347" s="4"/>
+    </row>
+    <row r="1348" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1348" s="4" t="s">
+        <v>3383</v>
+      </c>
+      <c r="B1348" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1348" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1348" s="4" t="s">
+        <v>3033</v>
+      </c>
+      <c r="E1348" s="4"/>
+      <c r="F1348" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1348" s="4" t="s">
+        <v>3380</v>
+      </c>
+      <c r="H1348" s="4"/>
+      <c r="I1348" s="4" t="s">
+        <v>3381</v>
+      </c>
+      <c r="J1348" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1348" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1348" s="4"/>
+    </row>
+    <row r="1349" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1349" s="4" t="s">
+        <v>3384</v>
+      </c>
+      <c r="B1349" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1349" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1349" s="4" t="s">
+        <v>2218</v>
+      </c>
+      <c r="E1349" s="4"/>
+      <c r="F1349" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1349" s="4" t="s">
+        <v>3380</v>
+      </c>
+      <c r="H1349" s="4"/>
+      <c r="I1349" s="4" t="s">
+        <v>3381</v>
+      </c>
+      <c r="J1349" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1349" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1349" s="4"/>
+    </row>
+    <row r="1350" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1350" s="4" t="s">
+        <v>3385</v>
+      </c>
+      <c r="B1350" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1350" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1350" s="4" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E1350" s="4"/>
+      <c r="F1350" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1350" s="4" t="s">
+        <v>3380</v>
+      </c>
+      <c r="H1350" s="4"/>
+      <c r="I1350" s="4" t="s">
+        <v>3381</v>
+      </c>
+      <c r="J1350" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1350" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1350" s="4"/>
+    </row>
+    <row r="1351" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1351" s="4" t="s">
+        <v>3386</v>
+      </c>
+      <c r="B1351" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1351" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1351" s="4" t="s">
+        <v>3387</v>
+      </c>
+      <c r="E1351" s="4"/>
+      <c r="F1351" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1351" s="4" t="s">
+        <v>3380</v>
+      </c>
+      <c r="H1351" s="4"/>
+      <c r="I1351" s="4" t="s">
+        <v>3381</v>
+      </c>
+      <c r="J1351" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1351" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1351" s="4"/>
+    </row>
+    <row r="1352" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1352" s="4" t="s">
+        <v>3388</v>
+      </c>
+      <c r="B1352" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1352" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1352" s="4" t="s">
+        <v>3387</v>
+      </c>
+      <c r="E1352" s="4"/>
+      <c r="F1352" s="4" t="s">
+        <v>700</v>
+      </c>
+      <c r="G1352" s="4" t="s">
+        <v>3389</v>
+      </c>
+      <c r="H1352" s="4"/>
+      <c r="I1352" s="4" t="s">
+        <v>3381</v>
+      </c>
+      <c r="J1352" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1352" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1352" s="4"/>
+    </row>
+    <row r="1353" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1353" s="4" t="s">
+        <v>3390</v>
+      </c>
+      <c r="B1353" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1353" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1353" s="4" t="s">
+        <v>2335</v>
+      </c>
+      <c r="E1353" s="4"/>
+      <c r="F1353" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1353" s="4" t="s">
+        <v>3380</v>
+      </c>
+      <c r="H1353" s="4"/>
+      <c r="I1353" s="4" t="s">
+        <v>3381</v>
+      </c>
+      <c r="J1353" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1353" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1353" s="4"/>
+    </row>
+    <row r="1354" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1354" s="4" t="s">
+        <v>3391</v>
+      </c>
+      <c r="B1354" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1354" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1354" s="4" t="s">
+        <v>2402</v>
+      </c>
+      <c r="E1354" s="4"/>
+      <c r="F1354" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1354" s="4" t="s">
+        <v>3380</v>
+      </c>
+      <c r="H1354" s="4"/>
+      <c r="I1354" s="4" t="s">
+        <v>3381</v>
+      </c>
+      <c r="J1354" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1354" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1354" s="4"/>
+    </row>
+    <row r="1355" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1355" s="4" t="s">
+        <v>3392</v>
+      </c>
+      <c r="B1355" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1355" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1355" s="4" t="s">
+        <v>3393</v>
+      </c>
+      <c r="E1355" s="4"/>
+      <c r="F1355" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1355" s="4" t="s">
+        <v>3380</v>
+      </c>
+      <c r="H1355" s="4"/>
+      <c r="I1355" s="4" t="s">
+        <v>3381</v>
+      </c>
+      <c r="J1355" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1355" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1355" s="4"/>
+    </row>
+    <row r="1356" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1356" s="4" t="s">
+        <v>3394</v>
+      </c>
+      <c r="B1356" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1356" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1356" s="4" t="s">
+        <v>3393</v>
+      </c>
+      <c r="E1356" s="4"/>
+      <c r="F1356" s="4" t="s">
+        <v>700</v>
+      </c>
+      <c r="G1356" s="4" t="s">
+        <v>3395</v>
+      </c>
+      <c r="H1356" s="4"/>
+      <c r="I1356" s="4" t="s">
+        <v>3381</v>
+      </c>
+      <c r="J1356" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1356" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1356" s="4"/>
+    </row>
+    <row r="1357" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1357" s="4" t="s">
+        <v>3396</v>
+      </c>
+      <c r="B1357" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1357" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1357" s="4" t="s">
+        <v>2425</v>
+      </c>
+      <c r="E1357" s="4"/>
+      <c r="F1357" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1357" s="4" t="s">
+        <v>3380</v>
+      </c>
+      <c r="H1357" s="4"/>
+      <c r="I1357" s="4" t="s">
+        <v>3381</v>
+      </c>
+      <c r="J1357" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1357" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1357" s="4"/>
+    </row>
+    <row r="1358" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1358" s="4" t="s">
+        <v>3397</v>
+      </c>
+      <c r="B1358" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1358" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1358" s="4" t="s">
+        <v>3398</v>
+      </c>
+      <c r="E1358" s="4"/>
+      <c r="F1358" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1358" s="4" t="s">
+        <v>3380</v>
+      </c>
+      <c r="H1358" s="4"/>
+      <c r="I1358" s="4" t="s">
+        <v>3381</v>
+      </c>
+      <c r="J1358" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1358" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1358" s="4"/>
+    </row>
+    <row r="1359" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1359" s="4" t="s">
+        <v>3399</v>
+      </c>
+      <c r="B1359" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1359" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1359" s="4" t="s">
+        <v>3398</v>
+      </c>
+      <c r="E1359" s="4"/>
+      <c r="F1359" s="4" t="s">
+        <v>700</v>
+      </c>
+      <c r="G1359" s="4" t="s">
+        <v>3400</v>
+      </c>
+      <c r="H1359" s="4" t="s">
+        <v>3401</v>
+      </c>
+      <c r="I1359" s="4" t="s">
+        <v>3381</v>
+      </c>
+      <c r="J1359" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1359" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1359" s="4" t="s">
+        <v>3402</v>
+      </c>
+    </row>
+    <row r="1360" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1360" s="4" t="s">
+        <v>3403</v>
+      </c>
+      <c r="B1360" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1360" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1360" s="4" t="s">
+        <v>2137</v>
+      </c>
+      <c r="E1360" s="4"/>
+      <c r="F1360" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1360" s="4" t="s">
+        <v>3404</v>
+      </c>
+      <c r="H1360" s="4"/>
+      <c r="I1360" s="4" t="s">
+        <v>3405</v>
+      </c>
+      <c r="J1360" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1360" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1360" s="4"/>
+    </row>
+    <row r="1361" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1361" s="4" t="s">
+        <v>3406</v>
+      </c>
+      <c r="B1361" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1361" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1361" s="4" t="s">
+        <v>2238</v>
+      </c>
+      <c r="E1361" s="4"/>
+      <c r="F1361" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1361" s="4" t="s">
+        <v>3404</v>
+      </c>
+      <c r="H1361" s="4"/>
+      <c r="I1361" s="4" t="s">
+        <v>3405</v>
+      </c>
+      <c r="J1361" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1361" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1361" s="4"/>
+    </row>
+    <row r="1362" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1362" s="4" t="s">
+        <v>3407</v>
+      </c>
+      <c r="B1362" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1362" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1362" s="4" t="s">
+        <v>2388</v>
+      </c>
+      <c r="E1362" s="4"/>
+      <c r="F1362" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1362" s="4" t="s">
+        <v>3404</v>
+      </c>
+      <c r="H1362" s="4"/>
+      <c r="I1362" s="4" t="s">
+        <v>3405</v>
+      </c>
+      <c r="J1362" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1362" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1362" s="4"/>
+    </row>
+    <row r="1363" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1363" s="4" t="s">
+        <v>3408</v>
+      </c>
+      <c r="B1363" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1363" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1363" s="4" t="s">
+        <v>3409</v>
+      </c>
+      <c r="E1363" s="4"/>
+      <c r="F1363" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1363" s="4" t="s">
+        <v>3404</v>
+      </c>
+      <c r="H1363" s="4"/>
+      <c r="I1363" s="4" t="s">
+        <v>3405</v>
+      </c>
+      <c r="J1363" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1363" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1363" s="4"/>
+    </row>
+    <row r="1364" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1364" s="4" t="s">
+        <v>3410</v>
+      </c>
+      <c r="B1364" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1364" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1364" s="4" t="s">
+        <v>3409</v>
+      </c>
+      <c r="E1364" s="4"/>
+      <c r="F1364" s="4" t="s">
+        <v>700</v>
+      </c>
+      <c r="G1364" s="4" t="s">
+        <v>2950</v>
+      </c>
+      <c r="H1364" s="4"/>
+      <c r="I1364" s="4" t="s">
+        <v>3405</v>
+      </c>
+      <c r="J1364" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1364" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1364" s="4"/>
+    </row>
+    <row r="1365" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1365" s="4" t="s">
+        <v>3411</v>
+      </c>
+      <c r="B1365" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1365" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1365" s="4" t="s">
+        <v>2948</v>
+      </c>
+      <c r="E1365" s="4"/>
+      <c r="F1365" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1365" s="4" t="s">
+        <v>3404</v>
+      </c>
+      <c r="H1365" s="4"/>
+      <c r="I1365" s="4" t="s">
+        <v>3405</v>
+      </c>
+      <c r="J1365" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1365" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1365" s="4"/>
+    </row>
+    <row r="1366" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1366" s="4" t="s">
+        <v>3412</v>
+      </c>
+      <c r="B1366" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1366" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1366" s="4" t="s">
+        <v>2137</v>
+      </c>
+      <c r="E1366" s="4"/>
+      <c r="F1366" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1366" s="4" t="s">
+        <v>3413</v>
+      </c>
+      <c r="H1366" s="4"/>
+      <c r="I1366" s="4" t="s">
+        <v>3414</v>
+      </c>
+      <c r="J1366" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1366" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1366" s="4"/>
+    </row>
+    <row r="1367" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1367" s="4" t="s">
+        <v>3415</v>
+      </c>
+      <c r="B1367" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1367" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1367" s="4" t="s">
+        <v>2238</v>
+      </c>
+      <c r="E1367" s="4"/>
+      <c r="F1367" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1367" s="4" t="s">
+        <v>3413</v>
+      </c>
+      <c r="H1367" s="4"/>
+      <c r="I1367" s="4" t="s">
+        <v>3414</v>
+      </c>
+      <c r="J1367" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1367" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1367" s="4"/>
+    </row>
+    <row r="1368" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1368" s="4" t="s">
+        <v>3416</v>
+      </c>
+      <c r="B1368" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1368" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1368" s="4" t="s">
+        <v>2388</v>
+      </c>
+      <c r="E1368" s="4"/>
+      <c r="F1368" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1368" s="4" t="s">
+        <v>3413</v>
+      </c>
+      <c r="H1368" s="4"/>
+      <c r="I1368" s="4" t="s">
+        <v>3414</v>
+      </c>
+      <c r="J1368" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1368" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1368" s="4"/>
+    </row>
+    <row r="1369" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1369" s="4" t="s">
+        <v>3417</v>
+      </c>
+      <c r="B1369" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1369" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1369" s="4" t="s">
+        <v>2478</v>
+      </c>
+      <c r="E1369" s="4"/>
+      <c r="F1369" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1369" s="4" t="s">
+        <v>3413</v>
+      </c>
+      <c r="H1369" s="4"/>
+      <c r="I1369" s="4" t="s">
+        <v>3414</v>
+      </c>
+      <c r="J1369" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1369" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1369" s="4"/>
+    </row>
+    <row r="1370" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1370" s="4" t="s">
+        <v>3418</v>
+      </c>
+      <c r="B1370" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1370" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1370" s="4" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E1370" s="4"/>
+      <c r="F1370" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1370" s="4" t="s">
+        <v>3419</v>
+      </c>
+      <c r="H1370" s="4"/>
+      <c r="I1370" s="4" t="s">
+        <v>3420</v>
+      </c>
+      <c r="J1370" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1370" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1370" s="4"/>
+    </row>
+    <row r="1371" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1371" s="4" t="s">
+        <v>3421</v>
+      </c>
+      <c r="B1371" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1371" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1371" s="4" t="s">
+        <v>1837</v>
+      </c>
+      <c r="E1371" s="4"/>
+      <c r="F1371" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1371" s="4" t="s">
+        <v>3422</v>
+      </c>
+      <c r="H1371" s="4"/>
+      <c r="I1371" s="4" t="s">
+        <v>3423</v>
+      </c>
+      <c r="J1371" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1371" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1371" s="4"/>
+    </row>
+    <row r="1372" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1372" s="4" t="s">
+        <v>3424</v>
+      </c>
+      <c r="B1372" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1372" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1372" s="4" t="s">
+        <v>1704</v>
+      </c>
+      <c r="E1372" s="4"/>
+      <c r="F1372" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1372" s="4" t="s">
+        <v>3425</v>
+      </c>
+      <c r="H1372" s="4"/>
+      <c r="I1372" s="4" t="s">
+        <v>3426</v>
+      </c>
+      <c r="J1372" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1372" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1372" s="4"/>
+    </row>
+    <row r="1373" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1373" s="4" t="s">
+        <v>3427</v>
+      </c>
+      <c r="B1373" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1373" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1373" s="4" t="s">
+        <v>1727</v>
+      </c>
+      <c r="E1373" s="4"/>
+      <c r="F1373" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1373" s="4" t="s">
+        <v>3425</v>
+      </c>
+      <c r="H1373" s="4"/>
+      <c r="I1373" s="4" t="s">
+        <v>3426</v>
+      </c>
+      <c r="J1373" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1373" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1373" s="4"/>
+    </row>
+    <row r="1374" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1374" s="4" t="s">
+        <v>3428</v>
+      </c>
+      <c r="B1374" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1374" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1374" s="4" t="s">
+        <v>1751</v>
+      </c>
+      <c r="E1374" s="4"/>
+      <c r="F1374" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1374" s="4" t="s">
+        <v>3425</v>
+      </c>
+      <c r="H1374" s="4"/>
+      <c r="I1374" s="4" t="s">
+        <v>3426</v>
+      </c>
+      <c r="J1374" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1374" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1374" s="4"/>
+    </row>
+    <row r="1375" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1375" s="4" t="s">
+        <v>3429</v>
+      </c>
+      <c r="B1375" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1375" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1375" s="4" t="s">
+        <v>1773</v>
+      </c>
+      <c r="E1375" s="4"/>
+      <c r="F1375" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1375" s="4" t="s">
+        <v>3425</v>
+      </c>
+      <c r="H1375" s="4"/>
+      <c r="I1375" s="4" t="s">
+        <v>3426</v>
+      </c>
+      <c r="J1375" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1375" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1375" s="4"/>
+    </row>
+    <row r="1376" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1376" s="4" t="s">
+        <v>3430</v>
+      </c>
+      <c r="B1376" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1376" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1376" s="4" t="s">
+        <v>1826</v>
+      </c>
+      <c r="E1376" s="4"/>
+      <c r="F1376" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1376" s="4" t="s">
+        <v>3425</v>
+      </c>
+      <c r="H1376" s="4"/>
+      <c r="I1376" s="4" t="s">
+        <v>3426</v>
+      </c>
+      <c r="J1376" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1376" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1376" s="4"/>
+    </row>
+    <row r="1377" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1377" s="4" t="s">
+        <v>3431</v>
+      </c>
+      <c r="B1377" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1377" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1377" s="4" t="s">
+        <v>1968</v>
+      </c>
+      <c r="E1377" s="4"/>
+      <c r="F1377" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1377" s="4" t="s">
+        <v>3425</v>
+      </c>
+      <c r="H1377" s="4"/>
+      <c r="I1377" s="4" t="s">
+        <v>3426</v>
+      </c>
+      <c r="J1377" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1377" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1377" s="4"/>
+    </row>
+    <row r="1378" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1378" s="4" t="s">
+        <v>3432</v>
+      </c>
+      <c r="B1378" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1378" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1378" s="4" t="s">
+        <v>2045</v>
+      </c>
+      <c r="E1378" s="4"/>
+      <c r="F1378" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1378" s="4" t="s">
+        <v>3425</v>
+      </c>
+      <c r="H1378" s="4"/>
+      <c r="I1378" s="4" t="s">
+        <v>3426</v>
+      </c>
+      <c r="J1378" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1378" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1378" s="4"/>
+    </row>
+    <row r="1379" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1379" s="4" t="s">
+        <v>3433</v>
+      </c>
+      <c r="B1379" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1379" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1379" s="4" t="s">
+        <v>2087</v>
+      </c>
+      <c r="E1379" s="4"/>
+      <c r="F1379" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1379" s="4" t="s">
+        <v>3425</v>
+      </c>
+      <c r="H1379" s="4"/>
+      <c r="I1379" s="4" t="s">
+        <v>3426</v>
+      </c>
+      <c r="J1379" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1379" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1379" s="4"/>
+    </row>
+    <row r="1380" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1380" s="4" t="s">
+        <v>3434</v>
+      </c>
+      <c r="B1380" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1380" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1380" s="4" t="s">
+        <v>2103</v>
+      </c>
+      <c r="E1380" s="4"/>
+      <c r="F1380" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1380" s="4" t="s">
+        <v>3425</v>
+      </c>
+      <c r="H1380" s="4"/>
+      <c r="I1380" s="4" t="s">
+        <v>3426</v>
+      </c>
+      <c r="J1380" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1380" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1380" s="4"/>
+    </row>
+    <row r="1381" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1381" s="4" t="s">
+        <v>3435</v>
+      </c>
+      <c r="B1381" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1381" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1381" s="4" t="s">
+        <v>1723</v>
+      </c>
+      <c r="E1381" s="4"/>
+      <c r="F1381" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1381" s="4" t="s">
+        <v>3436</v>
+      </c>
+      <c r="H1381" s="4"/>
+      <c r="I1381" s="4" t="s">
+        <v>3437</v>
+      </c>
+      <c r="J1381" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1381" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1381" s="4"/>
+    </row>
+    <row r="1382" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1382" s="4" t="s">
+        <v>3438</v>
+      </c>
+      <c r="B1382" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1382" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1382" s="4" t="s">
+        <v>1731</v>
+      </c>
+      <c r="E1382" s="4"/>
+      <c r="F1382" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1382" s="4" t="s">
+        <v>3436</v>
+      </c>
+      <c r="H1382" s="4"/>
+      <c r="I1382" s="4" t="s">
+        <v>3437</v>
+      </c>
+      <c r="J1382" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1382" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1382" s="4"/>
+    </row>
+    <row r="1383" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1383" s="4" t="s">
+        <v>3439</v>
+      </c>
+      <c r="B1383" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1383" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1383" s="4" t="s">
+        <v>1777</v>
+      </c>
+      <c r="E1383" s="4"/>
+      <c r="F1383" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1383" s="4" t="s">
+        <v>3436</v>
+      </c>
+      <c r="H1383" s="4"/>
+      <c r="I1383" s="4" t="s">
+        <v>3437</v>
+      </c>
+      <c r="J1383" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1383" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1383" s="4"/>
+    </row>
+    <row r="1384" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1384" s="4" t="s">
+        <v>3440</v>
+      </c>
+      <c r="B1384" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1384" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1384" s="4" t="s">
+        <v>1787</v>
+      </c>
+      <c r="E1384" s="4"/>
+      <c r="F1384" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1384" s="4" t="s">
+        <v>3436</v>
+      </c>
+      <c r="H1384" s="4"/>
+      <c r="I1384" s="4" t="s">
+        <v>3437</v>
+      </c>
+      <c r="J1384" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1384" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1384" s="4"/>
+    </row>
+    <row r="1385" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1385" s="4" t="s">
+        <v>3441</v>
+      </c>
+      <c r="B1385" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1385" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1385" s="4" t="s">
+        <v>2028</v>
+      </c>
+      <c r="E1385" s="4"/>
+      <c r="F1385" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1385" s="4" t="s">
+        <v>3436</v>
+      </c>
+      <c r="H1385" s="4"/>
+      <c r="I1385" s="4" t="s">
+        <v>3437</v>
+      </c>
+      <c r="J1385" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1385" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1385" s="4"/>
+    </row>
+    <row r="1386" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1386" s="4" t="s">
+        <v>3442</v>
+      </c>
+      <c r="B1386" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1386" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1386" s="4" t="s">
+        <v>2063</v>
+      </c>
+      <c r="E1386" s="4"/>
+      <c r="F1386" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1386" s="4" t="s">
+        <v>3436</v>
+      </c>
+      <c r="H1386" s="4"/>
+      <c r="I1386" s="4" t="s">
+        <v>3437</v>
+      </c>
+      <c r="J1386" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1386" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1386" s="4"/>
+    </row>
+    <row r="1387" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1387" s="4" t="s">
+        <v>3443</v>
+      </c>
+      <c r="B1387" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1387" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1387" s="4" t="s">
+        <v>1984</v>
+      </c>
+      <c r="E1387" s="4"/>
+      <c r="F1387" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1387" s="4" t="s">
+        <v>3425</v>
+      </c>
+      <c r="H1387" s="4"/>
+      <c r="I1387" s="4" t="s">
+        <v>3444</v>
+      </c>
+      <c r="J1387" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1387" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1387" s="4" t="s">
+        <v>3445</v>
+      </c>
+    </row>
+    <row r="1388" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1388" s="4" t="s">
+        <v>3446</v>
+      </c>
+      <c r="B1388" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C1388" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1388" s="4" t="s">
+        <v>1636</v>
+      </c>
+      <c r="E1388" s="4"/>
+      <c r="F1388" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="G1388" s="4" t="s">
+        <v>3447</v>
+      </c>
+      <c r="H1388" s="4"/>
+      <c r="I1388" s="4" t="s">
+        <v>3448</v>
+      </c>
+      <c r="J1388" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="K1388" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="L1388" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -56900,25 +58714,25 @@
   <dimension ref="A1:F17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>3369</v>
+        <v>3449</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>3370</v>
+        <v>3450</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>3371</v>
+        <v>3451</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>3372</v>
+        <v>3452</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>696</v>
@@ -56927,9 +58741,9 @@
         <v>647</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>3373</v>
+        <v>3453</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>905</v>
@@ -56938,18 +58752,18 @@
         <v>860</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>3374</v>
+        <v>3454</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>3375</v>
+        <v>3455</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>669</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>3376</v>
+        <v>3456</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>1008</v>
@@ -56958,18 +58772,18 @@
         <v>1056</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>3374</v>
+        <v>3454</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>3377</v>
+        <v>3457</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>669</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>3378</v>
+        <v>3458</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>1138</v>
@@ -56978,18 +58792,18 @@
         <v>1151</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>3374</v>
+        <v>3454</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>3379</v>
+        <v>3459</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>669</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>3380</v>
+        <v>3460</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>1207</v>
@@ -56998,112 +58812,112 @@
         <v>990</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>3374</v>
+        <v>3454</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>3381</v>
+        <v>3461</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>669</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>3382</v>
+        <v>3462</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>1143</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>3383</v>
+        <v>3463</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>3374</v>
+        <v>3454</v>
       </c>
       <c r="E6" s="4"/>
       <c r="F6" s="4" t="s">
         <v>669</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>3384</v>
+        <v>3464</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>3385</v>
+        <v>3465</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>913</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>3374</v>
+        <v>3454</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>3386</v>
+        <v>3466</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>669</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>3387</v>
+        <v>3467</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>3385</v>
+        <v>3465</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>3388</v>
+        <v>3468</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>3389</v>
+        <v>3469</v>
       </c>
       <c r="E8" s="4"/>
       <c r="F8" s="4" t="s">
         <v>669</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>3390</v>
+        <v>3470</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>1196</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>3391</v>
+        <v>3471</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>3392</v>
+        <v>3472</v>
       </c>
       <c r="E9" s="4"/>
       <c r="F9" s="4" t="s">
         <v>669</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>3393</v>
+        <v>3473</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>3394</v>
+        <v>3474</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>848</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>3374</v>
+        <v>3454</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>3395</v>
+        <v>3475</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>669</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>3396</v>
+        <v>3476</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>930</v>
@@ -57112,18 +58926,18 @@
         <v>1263</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>3374</v>
+        <v>3454</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>3397</v>
+        <v>3477</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>669</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>3398</v>
+        <v>3478</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>1114</v>
@@ -57132,18 +58946,18 @@
         <v>786</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>3374</v>
+        <v>3454</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>3399</v>
+        <v>3479</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>669</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>3400</v>
+        <v>3480</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>1228</v>
@@ -57152,16 +58966,16 @@
         <v>768</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>3374</v>
+        <v>3454</v>
       </c>
       <c r="E13" s="4"/>
       <c r="F13" s="4" t="s">
         <v>669</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>3401</v>
+        <v>3481</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>2437</v>
@@ -57170,36 +58984,36 @@
         <v>2434</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>3374</v>
+        <v>3454</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>3402</v>
+        <v>3482</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>669</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>3403</v>
+        <v>3483</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>3404</v>
+        <v>3484</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>2828</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>3405</v>
+        <v>3485</v>
       </c>
       <c r="E15" s="4"/>
       <c r="F15" s="4" t="s">
         <v>669</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>3406</v>
+        <v>3486</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>1504</v>
@@ -57208,18 +59022,18 @@
         <v>2345</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>3407</v>
+        <v>3487</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>3408</v>
+        <v>3488</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>669</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>3409</v>
+        <v>3489</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>108</v>
@@ -57228,10 +59042,10 @@
         <v>2018</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>3410</v>
+        <v>3490</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>3411</v>
+        <v>3491</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>669</v>

</xml_diff>

<commit_message>
Tupuna-to-tupuna links (kin), waka links, whakapapa collection with union map view
</commit_message>
<xml_diff>
--- a/TKM_Iwi_Hapu_Marae_Database.xlsx
+++ b/TKM_Iwi_Hapu_Marae_Database.xlsx
@@ -114,7 +114,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Links a tupuna to any number of locations of interest. location_type: Marae | Hapū | Iwi | Place. location_ref: the marae/hapū/iwi name exactly as on the map, or a label for a Place. location_detail: for marae, the Location text as shown on the map (disambiguates same-name marae). latitude/longitude: only for Place. relationship: Born | Lived | Died | Buried | Affiliated | Land interest | Other.</t>
+          <t xml:space="preserve">Links a tupuna to any number of locations of interest OR to another tupuna. location_type: Marae | Hapū | Iwi | Waka | Place | Tupuna. location_ref: the marae/hapū/iwi/waka name as on the map, a label for a Place, or the other tupuna's tupuna_id (location_detail = their name). latitude/longitude: Place only. relationship — for locations: Born | Lived | Died | Buried | Affiliated | Land interest | Other; for Tupuna: Mother | Father | Child | Spouse / partner | Sibling | Grandparent | Grandchild | Ancestor | Descendant | Whāngai | Other (recorded from this tupuna's point of view; the map shows the inverse on the other card).</t>
         </r>
       </text>
     </comment>
@@ -57117,7 +57117,7 @@
       </c>
       <c r="L1339" s="4"/>
     </row>
-    <row r="1340" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1340" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1340" s="4" t="s">
         <v>3369</v>
       </c>
@@ -57149,7 +57149,7 @@
       </c>
       <c r="L1340" s="4"/>
     </row>
-    <row r="1341" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1341" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1341" s="4" t="s">
         <v>3372</v>
       </c>
@@ -57181,7 +57181,7 @@
       </c>
       <c r="L1341" s="4"/>
     </row>
-    <row r="1342" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1342" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1342" s="4" t="s">
         <v>3373</v>
       </c>
@@ -57213,7 +57213,7 @@
       </c>
       <c r="L1342" s="4"/>
     </row>
-    <row r="1343" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1343" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1343" s="4" t="s">
         <v>3375</v>
       </c>
@@ -57245,7 +57245,7 @@
       </c>
       <c r="L1343" s="4"/>
     </row>
-    <row r="1344" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1344" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1344" s="4" t="s">
         <v>3376</v>
       </c>
@@ -57277,7 +57277,7 @@
       </c>
       <c r="L1344" s="4"/>
     </row>
-    <row r="1345" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1345" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1345" s="4" t="s">
         <v>3377</v>
       </c>
@@ -57309,7 +57309,7 @@
       </c>
       <c r="L1345" s="4"/>
     </row>
-    <row r="1346" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1346" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1346" s="4" t="s">
         <v>3378</v>
       </c>
@@ -57341,7 +57341,7 @@
       </c>
       <c r="L1346" s="4"/>
     </row>
-    <row r="1347" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1347" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1347" s="4" t="s">
         <v>3382</v>
       </c>
@@ -57373,7 +57373,7 @@
       </c>
       <c r="L1347" s="4"/>
     </row>
-    <row r="1348" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1348" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1348" s="4" t="s">
         <v>3383</v>
       </c>
@@ -57405,7 +57405,7 @@
       </c>
       <c r="L1348" s="4"/>
     </row>
-    <row r="1349" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1349" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1349" s="4" t="s">
         <v>3384</v>
       </c>
@@ -57437,7 +57437,7 @@
       </c>
       <c r="L1349" s="4"/>
     </row>
-    <row r="1350" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1350" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1350" s="4" t="s">
         <v>3385</v>
       </c>
@@ -57469,7 +57469,7 @@
       </c>
       <c r="L1350" s="4"/>
     </row>
-    <row r="1351" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1351" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1351" s="4" t="s">
         <v>3386</v>
       </c>
@@ -57501,7 +57501,7 @@
       </c>
       <c r="L1351" s="4"/>
     </row>
-    <row r="1352" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1352" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1352" s="4" t="s">
         <v>3388</v>
       </c>
@@ -57533,7 +57533,7 @@
       </c>
       <c r="L1352" s="4"/>
     </row>
-    <row r="1353" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1353" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1353" s="4" t="s">
         <v>3390</v>
       </c>
@@ -57565,7 +57565,7 @@
       </c>
       <c r="L1353" s="4"/>
     </row>
-    <row r="1354" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1354" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1354" s="4" t="s">
         <v>3391</v>
       </c>
@@ -57597,7 +57597,7 @@
       </c>
       <c r="L1354" s="4"/>
     </row>
-    <row r="1355" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1355" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1355" s="4" t="s">
         <v>3392</v>
       </c>
@@ -57629,7 +57629,7 @@
       </c>
       <c r="L1355" s="4"/>
     </row>
-    <row r="1356" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1356" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1356" s="4" t="s">
         <v>3394</v>
       </c>
@@ -57661,7 +57661,7 @@
       </c>
       <c r="L1356" s="4"/>
     </row>
-    <row r="1357" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1357" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1357" s="4" t="s">
         <v>3396</v>
       </c>
@@ -57693,7 +57693,7 @@
       </c>
       <c r="L1357" s="4"/>
     </row>
-    <row r="1358" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1358" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1358" s="4" t="s">
         <v>3397</v>
       </c>
@@ -57725,7 +57725,7 @@
       </c>
       <c r="L1358" s="4"/>
     </row>
-    <row r="1359" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1359" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1359" s="4" t="s">
         <v>3399</v>
       </c>
@@ -57761,7 +57761,7 @@
         <v>3402</v>
       </c>
     </row>
-    <row r="1360" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1360" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1360" s="4" t="s">
         <v>3403</v>
       </c>
@@ -57793,7 +57793,7 @@
       </c>
       <c r="L1360" s="4"/>
     </row>
-    <row r="1361" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1361" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1361" s="4" t="s">
         <v>3406</v>
       </c>
@@ -57825,7 +57825,7 @@
       </c>
       <c r="L1361" s="4"/>
     </row>
-    <row r="1362" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1362" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1362" s="4" t="s">
         <v>3407</v>
       </c>
@@ -57857,7 +57857,7 @@
       </c>
       <c r="L1362" s="4"/>
     </row>
-    <row r="1363" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1363" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1363" s="4" t="s">
         <v>3408</v>
       </c>
@@ -57889,7 +57889,7 @@
       </c>
       <c r="L1363" s="4"/>
     </row>
-    <row r="1364" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1364" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1364" s="4" t="s">
         <v>3410</v>
       </c>
@@ -57921,7 +57921,7 @@
       </c>
       <c r="L1364" s="4"/>
     </row>
-    <row r="1365" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1365" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1365" s="4" t="s">
         <v>3411</v>
       </c>
@@ -57953,7 +57953,7 @@
       </c>
       <c r="L1365" s="4"/>
     </row>
-    <row r="1366" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1366" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1366" s="4" t="s">
         <v>3412</v>
       </c>
@@ -57985,7 +57985,7 @@
       </c>
       <c r="L1366" s="4"/>
     </row>
-    <row r="1367" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1367" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1367" s="4" t="s">
         <v>3415</v>
       </c>
@@ -58017,7 +58017,7 @@
       </c>
       <c r="L1367" s="4"/>
     </row>
-    <row r="1368" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1368" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1368" s="4" t="s">
         <v>3416</v>
       </c>
@@ -58049,7 +58049,7 @@
       </c>
       <c r="L1368" s="4"/>
     </row>
-    <row r="1369" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1369" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1369" s="4" t="s">
         <v>3417</v>
       </c>
@@ -58081,7 +58081,7 @@
       </c>
       <c r="L1369" s="4"/>
     </row>
-    <row r="1370" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1370" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1370" s="4" t="s">
         <v>3418</v>
       </c>
@@ -58113,7 +58113,7 @@
       </c>
       <c r="L1370" s="4"/>
     </row>
-    <row r="1371" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1371" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1371" s="4" t="s">
         <v>3421</v>
       </c>
@@ -58145,7 +58145,7 @@
       </c>
       <c r="L1371" s="4"/>
     </row>
-    <row r="1372" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1372" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1372" s="4" t="s">
         <v>3424</v>
       </c>
@@ -58177,7 +58177,7 @@
       </c>
       <c r="L1372" s="4"/>
     </row>
-    <row r="1373" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1373" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1373" s="4" t="s">
         <v>3427</v>
       </c>
@@ -58209,7 +58209,7 @@
       </c>
       <c r="L1373" s="4"/>
     </row>
-    <row r="1374" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1374" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1374" s="4" t="s">
         <v>3428</v>
       </c>
@@ -58241,7 +58241,7 @@
       </c>
       <c r="L1374" s="4"/>
     </row>
-    <row r="1375" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1375" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1375" s="4" t="s">
         <v>3429</v>
       </c>
@@ -58273,7 +58273,7 @@
       </c>
       <c r="L1375" s="4"/>
     </row>
-    <row r="1376" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1376" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1376" s="4" t="s">
         <v>3430</v>
       </c>
@@ -58305,7 +58305,7 @@
       </c>
       <c r="L1376" s="4"/>
     </row>
-    <row r="1377" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1377" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1377" s="4" t="s">
         <v>3431</v>
       </c>
@@ -58337,7 +58337,7 @@
       </c>
       <c r="L1377" s="4"/>
     </row>
-    <row r="1378" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1378" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1378" s="4" t="s">
         <v>3432</v>
       </c>
@@ -58369,7 +58369,7 @@
       </c>
       <c r="L1378" s="4"/>
     </row>
-    <row r="1379" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1379" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1379" s="4" t="s">
         <v>3433</v>
       </c>
@@ -58401,7 +58401,7 @@
       </c>
       <c r="L1379" s="4"/>
     </row>
-    <row r="1380" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1380" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1380" s="4" t="s">
         <v>3434</v>
       </c>
@@ -58433,7 +58433,7 @@
       </c>
       <c r="L1380" s="4"/>
     </row>
-    <row r="1381" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1381" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1381" s="4" t="s">
         <v>3435</v>
       </c>
@@ -58465,7 +58465,7 @@
       </c>
       <c r="L1381" s="4"/>
     </row>
-    <row r="1382" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1382" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1382" s="4" t="s">
         <v>3438</v>
       </c>
@@ -58497,7 +58497,7 @@
       </c>
       <c r="L1382" s="4"/>
     </row>
-    <row r="1383" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1383" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1383" s="4" t="s">
         <v>3439</v>
       </c>
@@ -58529,7 +58529,7 @@
       </c>
       <c r="L1383" s="4"/>
     </row>
-    <row r="1384" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1384" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1384" s="4" t="s">
         <v>3440</v>
       </c>
@@ -58561,7 +58561,7 @@
       </c>
       <c r="L1384" s="4"/>
     </row>
-    <row r="1385" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1385" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1385" s="4" t="s">
         <v>3441</v>
       </c>
@@ -58593,7 +58593,7 @@
       </c>
       <c r="L1385" s="4"/>
     </row>
-    <row r="1386" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1386" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1386" s="4" t="s">
         <v>3442</v>
       </c>
@@ -58625,7 +58625,7 @@
       </c>
       <c r="L1386" s="4"/>
     </row>
-    <row r="1387" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1387" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1387" s="4" t="s">
         <v>3443</v>
       </c>
@@ -58659,7 +58659,7 @@
         <v>3445</v>
       </c>
     </row>
-    <row r="1388" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1388" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1388" s="4" t="s">
         <v>3446</v>
       </c>

</xml_diff>